<commit_message>
Mise à jour renommage modèle métier 8016cfb642525dafa57dacb6089e2f633c02bcd5
</commit_message>
<xml_diff>
--- a/htr-Corps-ModeleMetier/ig/StructureDefinition-fr-lm-entete-document.xlsx
+++ b/htr-Corps-ModeleMetier/ig/StructureDefinition-fr-lm-entete-document.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-10-21T08:19:27+00:00</t>
+    <t>2025-10-21T12:36:21+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -386,7 +386,7 @@
     <t>fr-lm-entete-document.destinataire</t>
   </si>
   <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-destinataire-prevu-document
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-destinataire-prevu
 </t>
   </si>
   <si>
@@ -785,7 +785,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="81.80078125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="76.6640625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>

</xml_diff>